<commit_message>
Added variation of Sequential Joint - Seg First
</commit_message>
<xml_diff>
--- a/training_results.xlsx
+++ b/training_results.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\TFG\repo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94D71972-FB18-4172-A47F-A9AFBE7F84EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24921C28-B9D5-4FB2-ACAC-242EE2E27330}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="18">
   <si>
     <t>Dataset</t>
   </si>
@@ -71,14 +71,25 @@
   </si>
   <si>
     <t>Joint Combined</t>
+  </si>
+  <si>
+    <t>Sequential Joint</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -106,8 +117,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -410,11 +422,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="25.85546875" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:I15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -453,13 +462,13 @@
         <v>10</v>
       </c>
       <c r="C2">
-        <v>44.717117309570298</v>
+        <v>42.651275634765618</v>
       </c>
       <c r="D2">
-        <v>0.99043649435043302</v>
+        <v>0.98935848474502563</v>
       </c>
       <c r="E2">
-        <v>2.5815172120928699E-3</v>
+        <v>3.097000764682889E-3</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -470,16 +479,16 @@
         <v>11</v>
       </c>
       <c r="F3">
-        <v>0.62107735872268599</v>
+        <v>0.78211629390716553</v>
       </c>
       <c r="G3">
-        <v>0.68976253271102905</v>
+        <v>0.64219290018081665</v>
       </c>
       <c r="H3">
-        <v>0.95141983032226496</v>
+        <v>0.8341938853263855</v>
       </c>
       <c r="I3">
-        <v>0.92734134197235096</v>
+        <v>0.73615884780883789</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -490,16 +499,16 @@
         <v>12</v>
       </c>
       <c r="F4">
-        <v>0.689955294132232</v>
+        <v>0.79833734035491943</v>
       </c>
       <c r="G4">
-        <v>0.73864173889160101</v>
+        <v>0.6643606424331665</v>
       </c>
       <c r="H4">
-        <v>0.96011507511138905</v>
+        <v>0.85423839092254639</v>
       </c>
       <c r="I4">
-        <v>0.95079684257507302</v>
+        <v>0.74930328130722046</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -510,16 +519,16 @@
         <v>13</v>
       </c>
       <c r="F5">
-        <v>0.69951921701431197</v>
+        <v>0.80541235208511353</v>
       </c>
       <c r="G5">
-        <v>0.747727930545806</v>
+        <v>0.67421787977218628</v>
       </c>
       <c r="H5">
-        <v>0.95754826068878096</v>
+        <v>0.85476058721542358</v>
       </c>
       <c r="I5">
-        <v>0.94669628143310502</v>
+        <v>0.76145118474960327</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -530,16 +539,16 @@
         <v>14</v>
       </c>
       <c r="F6">
-        <v>0.83967983722686701</v>
+        <v>0.7942543625831604</v>
       </c>
       <c r="G6">
-        <v>0.87048506736755304</v>
+        <v>0.65872460603713989</v>
       </c>
       <c r="H6">
-        <v>0.978626668453216</v>
+        <v>0.87272465229034424</v>
       </c>
       <c r="I6">
-        <v>0.97577857971191395</v>
+        <v>0.72873109579086304</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -550,16 +559,16 @@
         <v>15</v>
       </c>
       <c r="F7">
-        <v>0.71284812688827504</v>
+        <v>0.79771530628204346</v>
       </c>
       <c r="G7">
-        <v>0.75501292943954401</v>
+        <v>0.66349953413009644</v>
       </c>
       <c r="H7">
-        <v>0.95671254396438599</v>
+        <v>0.86244726181030273</v>
       </c>
       <c r="I7">
-        <v>0.94809722900390603</v>
+        <v>0.74202203750610352</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -570,17 +579,40 @@
         <v>16</v>
       </c>
       <c r="F8">
-        <v>0.706021428108215</v>
+        <v>0.79566109180450439</v>
       </c>
       <c r="G8">
-        <v>0.75255739688873202</v>
+        <v>0.66066211462020874</v>
       </c>
       <c r="H8">
-        <v>0.95752453804016102</v>
+        <v>0.82313477993011475</v>
       </c>
       <c r="I8">
-        <v>0.94694471359252896</v>
-      </c>
+        <v>0.76996219158172607</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9">
+        <v>0.80309969186782804</v>
+      </c>
+      <c r="G9">
+        <v>0.67098295688629195</v>
+      </c>
+      <c r="H9">
+        <v>0.87370359897613503</v>
+      </c>
+      <c r="I9">
+        <v>0.74305367469787598</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I15" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>